<commit_message>
M5 in-run modifiers and economy
Engine: modifiers/hooks.ts hook points and modifiers/registry.ts with the
12-modifier subset (Suffix/Prefix Bias, Inflection, Vowel Harmony,
Coinage, Rack Extension, Momentum, Etymologist, Agglutination, Mirror,
Chain Lightning, Polyglot), folded in acquisition order and validated at
startup. Scoring gains per-morpheme values and a multiplier-base override.
economy.ts: round clear, margin bonus, natural streak, natural word
dividend, extension payout, Coinage, Bank; boss clear. reward.ts: boss
offers by rarity-per-boss odds and the conditional shop slot (D8).
Secret words flag a boss jump and an achievement. Streak breaks on card
use rather than strain.

UI: RewardScreen, ModifierPanel overlay, currency sources and modifier
notes on the score screen, in-run slot in the shop, modifier-aware
previews. Workbook: reward odds table added to the In-Run Modifiers tab.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -194,6 +194,9 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3431,7 +3434,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3727,7 +3729,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -3799,7 +3800,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -4195,7 +4195,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
@@ -4203,10 +4202,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4218,7 +4213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4241,6 +4236,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5244,6 +5240,161 @@
       <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Offer rules (proposal): after each boss, 3 random modifiers (4 with Bazaar L4 or Polyglot). Rarity odds shift toward Exotic/Relic in later bosses. Duplicates are not offered. Viewed in a dedicated In-Run Modifier panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Boss reward offer — rarity odds by boss (prototype values, [proposal])</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Exotic</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Relic</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C46" s="23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D46" s="23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E46" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D47" s="23" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E47" s="23" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C48" s="23" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D48" s="23" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E48" s="23" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C49" s="23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D49" s="23" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E49" s="23" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C50" s="23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D50" s="23" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E50" s="23" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C51" s="23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D51" s="23" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E51" s="23" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Offers: 3 (4 with Polyglot, which also picks 2). Never a modifier already held; no duplicates. The conditional shop slot offers Basic/Uncommon only (D8) for 10 currency.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M8: bot playtests and tuning pass 1
scripts/bot.ts plays runs through the real engine (extendability index
over the dictionary, greedy natural steps, extension cards when stuck,
greedy short words in boss rounds); scripts/playtest.ts writes seeded
reports with margins per round (npm run playtest). 10-seed baseline and
tuned reports in playtests/.

Tuning from the data: boss threshold factor 1.5 → 3 (boss score is
feed-bound); Agglutination +0.03, Momentum +0.01, Chain Lightning +0.02
(base bonuses are exponentiated); Extension guarantee limited to Hyphen,
Before & After, Free Morpheme. Workbook and scenario fixture updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -4632,12 +4632,12 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Each natural extension round adds a permanent +0.05 to the multiplier base.</t>
+          <t>Each natural extension round adds a permanent +0.01 to the multiplier base.</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Rewards abstaining from extension cards.</t>
+          <t>Rewards abstaining from extension cards. Was +0.05 — the base is exponentiated by morpheme count, so +0.05/round reached 2000× the threshold by round 22 in bot playtests.</t>
         </is>
       </c>
     </row>
@@ -4902,12 +4902,12 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Morpheme multiplier base +0.1.</t>
+          <t>Morpheme multiplier base +0.03.</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Everything.</t>
+          <t>Everything. Was +0.1 (see Momentum).</t>
         </is>
       </c>
     </row>
@@ -5118,12 +5118,12 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Extension cards grant +0.1 to the multiplier base instead of causing strain.</t>
+          <t>Extension cards grant +0.02 to the multiplier base instead of causing strain.</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Before &amp; After; Echo; Etymologist.</t>
+          <t>Before &amp; After; Echo; Etymologist. Was +0.1 (see Momentum).</t>
         </is>
       </c>
     </row>
@@ -5235,6 +5235,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="117" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
@@ -5242,6 +5243,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
@@ -7437,6 +7439,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7474,7 +7477,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Bazaar adds slots. Proposal: at least one Extension card is guaranteed if the player holds none.</t>
+          <t>Bazaar adds slots. The guaranteed Extension card (offered when the player holds none) is drawn from cards that work with any hand: Before &amp; After, Hyphen, Blend, Free Morpheme — Reduplication needs the exact tail letters and stranded runs in playtests.</t>
         </is>
       </c>
     </row>
@@ -7538,6 +7541,7 @@
       </c>
       <c r="C10" s="5" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -7630,6 +7634,7 @@
       </c>
       <c r="C19" s="7" t="n"/>
     </row>
+    <row r="20"/>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -8347,7 +8352,12 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1.5</v>
+        <v>3</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Raised from 1.5 after bot playtests (2026-09-16): boss score is feed-bound (~all fed tiles get placed), so 1.5 gave 6–12× margins. At 3 the scenario below still passes every boss with a narrowing margin (1.02–1.36 for B4–B6).</t>
+        </is>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Loadout budget grows per boss beaten
Each boss beaten in a run adds +1 loadout budget while the budget is
below that boss's cap (B1 6, B2 8, B3 10, B4 12, B5 14, B6 16), so
progression no longer depends on three achievements; achievements still
add on top up to 20. balance.meta.bossBudget; meta.applyRunEnd; awards
show the boss share; DESIGN.md rev 5; Pre-Run and Summary tabs updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -1170,7 +1170,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Shared points for tile modifiers (cost = level) and pre-run categories (cost = activated level). Grows with milestones; capped so choices stay strategic.</t>
+          <t>Shared points for tile modifiers (cost = level) and pre-run categories (cost = activated level). Starts at 4; grows +1 per boss beaten up to a per-boss cap (6 / 8 / 10 / 12 / 14 / 16 for B1–B6) and through achievements, hard cap 20.</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Loadout budget: shared between tile modifiers and pre-run categories. Grows with achievements/milestones. Proposal: hard cap of 20 base points (+ challenge points), and a cap of 8 modified letters. Prototype: the budget starts at 4 points [proposal]; positive-category levels are cumulative (L2 includes L1).</t>
+          <t>Loadout budget: shared between tile modifiers and pre-run categories. Starts at 4. Grows per boss beaten: each boss beaten in a run adds +1 while the budget is below that boss's cap — B1 → 6, B2 → 8, B3 → 10, B4 → 12, B5 → 14, B6 → 16 — so a player who cannot pass B3 tops out at 10. Achievements add on top, up to the hard cap of 20 (+ risk / challenge points). Cap of 8 modified letters. Positive-category levels are cumulative (L2 includes L1).</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5235,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="117" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
@@ -5243,7 +5242,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
@@ -7439,7 +7437,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7541,7 +7538,6 @@
       </c>
       <c r="C10" s="5" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -7634,7 +7630,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Undo covers card uses; inline confirms; Decisions tab
Sound Shifts and other card uses during a round now push undo snapshots
(kind 'card'); undo is LIFO over steps and cards so a shift that breaks
the word can be taken back. Forfeit and Reset progression used
window.confirm, which is blocked in the desktop app's browser pane and
made the buttons no-ops; replaced with an inline ConfirmButton.

Workbook: new Decisions tab with nine open/decided design calls, led by
the Sound Shift re-evaluation (a shift that invalidates the head word
cannot be repaired under back-only extension). DESIGN.md §7 item 9.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Boss Round Modifiers" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Scoring" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Achievements" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Decisions" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -148,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +197,9 @@
     <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2151,6 +2155,426 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Open design decisions raised by building and playtesting the prototype. Status: open / decided / dropped. When decided, update DESIGN.md and the relevant tab, and note the outcome here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Date raised</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Decision needed</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Context / evidence</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Cards — Sound Shift</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Re-evaluate Sound Shift cards. Once a shift makes the active word invalid, later steps must restore it — but back-only extension (D5) can never repair a broken head word, and a Before &amp; After moves the tail elsewhere, so the run gets stuck. Many shifts are therefore rarely usable.</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Playtest 2026-09-16: "prestaged" shifted to "rrestaged", then B&amp;A "do" → head "rrestaged" permanently invalid; SUBMIT rejected. Prototype fix: card uses are now undoable (Undo last card) so the player can recover, but the design question stands.</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>(a) Validate only the words a shift touches and allow front steps to repair the head. (b) Preview-and-reject: a shift is only allowed if the resulting word is valid or can be completed from the hand. (c) Shifts apply to the *next* step only (change letters of the tiles you are about to play). (d) Make shifts strain-free but require validity immediately (reject invalid shifts).</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Cards — Extension guarantee</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>Which cards may fill the guaranteed Extension slot?</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Reduplication and Blend stranded bot runs at round 3 (need specific tail letters).</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>Current prototype rule: Hyphen / Before &amp; After / Free Morpheme only (balance.shop.guaranteePool).</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>decided (prototype)</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>Pool limited to cards usable with any hand; revisit with human playtests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Scoring — boss factor</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Boss threshold factor: 1.5 → 3.</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Boss score is feed-bound (nearly every fed tile gets placed); at 1.5 the bot beat B1 by 7–37×. At 3 the Scoring-tab scenario still passes all bosses with narrowing margins (B4–B6: 1.36 / 1.42 / 1.08).</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Keep 3; or 2.5 if B3+ feel punishing to humans once the loadout budget reaches 8–10.</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>decided (prototype)</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>Factor 3 (Scoring tab C8). Watch B3–B6 in human playtests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Modifiers — base bonuses</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Magnitude of modifiers that add to the multiplier base.</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>The base is raised to (morphemes − 1): +0.1 / +0.05 per round reached 2000× the threshold by round 22 in bot runs.</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Agglutination +0.03, Momentum +0.01 per natural round, Chain Lightning +0.02 per card, Polysynthesis +0.015 (all implemented). Alternative: convert these to flat round-score multipliers.</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>decided (prototype)</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>Reduced values in the In-Run Modifiers tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Meta — starting pool</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Which cards and in-run modifiers are in the pool for a new player? Achievements unlock cards/modifiers, but nothing says what is locked at the start.</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Prototype records unlocks in MetaState but does not gate shop/reward pools.</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>(a) Everything available; achievements add nothing (drop those rewards). (b) A small starting pool per type; unlocks grow it. (c) Rarity-gated: Basic/Uncommon from the start, Exotic/Relic via unlocks.</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Shop — tile modifier action</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>The "apply a Level 1–2 modifier to a tile in hand" shop action: which tile does it target? The hand is empty in the shop.</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>Prototype offers add/remove tile only; Tile Smith card applies a modifier in the round instead.</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>(a) Target a pool tile by letter. (b) Keep the hand through the shop. (c) Drop the shop action; Tile Smith covers it.</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Economy — extension cards</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Is a 3-currency Hyphen every round too generous? Once a flexible extension card is in hand the "always extend" pressure mostly disappears.</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Bot with a Hyphen policy: 9/10 wins on the 12-modifier pool, 4/10 on the full pool. Income 7–25 per round vs 3-currency Basic cards.</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>(a) Raise strain for Hyphen to 3. (b) Price extension cards by use count. (c) Cap extension cards per boss cycle. (d) Leave; difficulty comes from bosses.</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Meta — loadout budget</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>How the loadout budget grows.</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>Only three achievements grew it; players stuck before B3 sat at 4 points.</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Implemented: +1 per boss beaten while below that boss's cap (6/8/10/12/14/16), plus achievements up to 20.</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>DESIGN.md §6.3 rev 5; Pre-Run tab note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>Cards — not implemented</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Homophone and Preview cards; Rhyme is approximated as "shares the last two letters"; Decay boss modifier; Lexicon Hint and Scavenger modifiers.</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>Homophone/Rhyme need pronunciation data; Preview needs feed reordering UI; Decay has no meaning while words score on placement; Scavenger needs boss tiles to flow back to the pool.</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Drop, redesign, or add a pronunciation list (e.g. CMUdict) for production.</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Threshold growth by block, Substrate reorder, lives replay the round
Threshold growth per round now rises in blocks of four rounds
(1.5 / 2 / 2.5 / 3 / 3.5 / 5) via balance.scoring.thresholdGrowthByBlock;
Scoring tab formulas use a growth table (G6:G11) with per-round growth
and base-threshold columns; scenario fixture regenerated (the no-modifier
scenario now fails at B2). Substrate levels: free redraw / hand +1 /
hand +1 + redraw / hand +2 + redraw. A failed round with a life (or
Insurance) reverts to the round start and is replayed with a fresh hand;
bosses re-roll their modifier. Playtest runner gained --growth.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Every round has a score threshold that rises geometrically, with a bump on Boss Rounds. Missing one costs a life (if any) or ends the run.</t>
+          <t>Every round has a score threshold. It grows per round by a factor that rises in blocks of four rounds (1.5× for rounds 1–4, 2× for 5–8, 2.5× for 9–12, 3× for 13–16, 3.5× for 17–20, 5× for 21–24), with a ×3 bump on Boss Rounds. Missing one costs a life — the round is then replayed — or ends the run.</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2569,6 +2569,126 @@
         </is>
       </c>
       <c r="H13" s="24" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>Scoring — threshold curve</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Threshold growth per round by block instead of a flat 1.5.</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Human playtests: multi-step rounds with a streak and stacked modifiers outgrew a 1.5 geometric curve and made bosses trivial. Bot (no synergies) now dies at rounds 8–12 on the new table and even on gentler tables (1.5/1.75/2/2.25/2.5/3 and 1.5/1.75/1.75/2/2/2.5); the no-modifier Scoring-tab scenario fails at B2. Human data needed.</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Implemented: 1.5 / 2 / 2.5 / 3 / 3.5 / 5 (Scoring tab G6:G11; editable live in the debug panel). Fallbacks to try if humans stall at B3–B4: 1.5/1.75/2/2.25/2.5/3.</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>decided (prototype)</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>Watch where humans stall; B4 = 2.05M and B6 = 192B need strong multiplier stacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>Pre-run — Substrate</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Hand size was a huge advantage; reorder the levels.</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Playtest feedback.</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Implemented: L1 free redraw; L2 hand +1; L3 hand +1 + redraw; L4 hand +2 + redraw.</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>Pre-Run tab row updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>Lives — replay the round</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>Losing a life (fail or forfeit) replays the same round instead of advancing.</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>Advancing made a forfeit a free skip; replaying makes a life a free re-roll of the hand (regular) or a new modifier (boss).</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Implemented: the failed round's steps and card uses are undone, tiles return, a fresh hand is drawn; bosses re-roll the modifier (D1).</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>DESIGN.md §2.1; Second Breath note.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3858,6 +3978,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3925,7 +4046,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>A life absorbs one failed threshold. Proposal: the round still counts as failed for streak, and no shop is offered.</t>
+          <t>A life absorbs one failed threshold and the round is replayed (regular: fresh hand, the word as it was before the round; boss: a new modifier). The round still counts as failed for the streak and no shop is offered.</t>
         </is>
       </c>
     </row>
@@ -3969,27 +4090,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>1 free redraw per round</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
           <t>Hand size +1</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Hand size +2</t>
-        </is>
-      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
+          <t>Hand +1, 1 free redraw per round</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
           <t>Hand +2, 1 free redraw per round</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Hand +3, 1 free redraw per round</t>
-        </is>
-      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Hand size drives how often a natural extension is possible.</t>
+          <t>Hand size drives how often a natural extension is possible — retuned 2026-09-18 (was +1/+2/+2+redraw/+3+redraw): a bigger hand was too strong, so the first level is the redraw.</t>
         </is>
       </c>
     </row>
@@ -4153,6 +4274,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -4224,6 +4346,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -4619,6 +4742,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
@@ -8680,7 +8804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8689,7 +8813,7 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="8"/>
+    <col width="8" customWidth="1" min="7" max="8"/>
     <col width="10" customWidth="1" min="9" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
@@ -8718,6 +8842,11 @@
           <t>Parameters</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Threshold growth per round, by block</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8733,6 +8862,16 @@
           <t>morpheme multiplier = base ^ (effective morphemes − 1)</t>
         </is>
       </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8748,20 +8887,34 @@
           <t>Lowered from 6 so an unmodified run nearly always reaches B1 (round 4 threshold 20).</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Threshold growth per round</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>1.5</v>
-      </c>
+          <t>Threshold growth per round (by block — table at F5:G11)</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>threshold = T1 × growth ^ (round − 1)</t>
-        </is>
+          <t>threshold(r) = T1 × Π growth(block of k) for k = 2..r; column R holds each round's growth, column S the running base. Changed 2026-09-18 from a flat 1.5 after human playtests: multi-step rounds plus streak modifiers outgrew a geometric 1.5.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>5–8</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -8778,6 +8931,14 @@
           <t>Raised from 1.5 after bot playtests (2026-09-16): boss score is feed-bound (~all fed tiles get placed), so 1.5 gave 6–12× margins. At 3 the scenario below still passes every boss with a narrowing margin (1.02–1.36 for B4–B6).</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>9–12</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8788,6 +8949,14 @@
       <c r="C9" s="15" t="n">
         <v>1</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>13–16</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8798,6 +8967,14 @@
       <c r="C10" s="15" t="n">
         <v>1.5</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>17–20</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8808,6 +8985,14 @@
       <c r="C11" s="15" t="n">
         <v>2</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>21–24</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8930,6 +9115,16 @@
       <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>Pass?</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Base threshold</t>
         </is>
       </c>
     </row>
@@ -8993,11 +9188,19 @@
         <v/>
       </c>
       <c r="P16" s="18">
-        <f>ROUND($C$6*$C$7^(A16-1)*IF(B16="Boss",$C$8,1),0)</f>
+        <f>ROUND(S16*IF(B16="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q16" s="16">
         <f>IF(O16&gt;=P16,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R16" s="18">
+        <f>INDEX($G$6:$G$11,INT((A16-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S16" s="18">
+        <f>$C$6</f>
         <v/>
       </c>
     </row>
@@ -9061,11 +9264,19 @@
         <v/>
       </c>
       <c r="P17" s="18">
-        <f>ROUND($C$6*$C$7^(A17-1)*IF(B17="Boss",$C$8,1),0)</f>
+        <f>ROUND(S17*IF(B17="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q17" s="16">
         <f>IF(O17&gt;=P17,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R17" s="18">
+        <f>INDEX($G$6:$G$11,INT((A17-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S17" s="18">
+        <f>S16*R17</f>
         <v/>
       </c>
     </row>
@@ -9129,11 +9340,19 @@
         <v/>
       </c>
       <c r="P18" s="18">
-        <f>ROUND($C$6*$C$7^(A18-1)*IF(B18="Boss",$C$8,1),0)</f>
+        <f>ROUND(S18*IF(B18="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q18" s="16">
         <f>IF(O18&gt;=P18,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R18" s="18">
+        <f>INDEX($G$6:$G$11,INT((A18-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S18" s="18">
+        <f>S17*R18</f>
         <v/>
       </c>
     </row>
@@ -9197,11 +9416,19 @@
         <v/>
       </c>
       <c r="P19" s="22">
-        <f>ROUND($C$6*$C$7^(A19-1)*IF(B19="Boss",$C$8,1),0)</f>
+        <f>ROUND(S19*IF(B19="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q19" s="20">
         <f>IF(O19&gt;=P19,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R19" s="22">
+        <f>INDEX($G$6:$G$11,INT((A19-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S19" s="22">
+        <f>S18*R19</f>
         <v/>
       </c>
     </row>
@@ -9265,11 +9492,19 @@
         <v/>
       </c>
       <c r="P20" s="18">
-        <f>ROUND($C$6*$C$7^(A20-1)*IF(B20="Boss",$C$8,1),0)</f>
+        <f>ROUND(S20*IF(B20="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q20" s="16">
         <f>IF(O20&gt;=P20,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R20" s="18">
+        <f>INDEX($G$6:$G$11,INT((A20-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S20" s="18">
+        <f>S19*R20</f>
         <v/>
       </c>
     </row>
@@ -9333,11 +9568,19 @@
         <v/>
       </c>
       <c r="P21" s="18">
-        <f>ROUND($C$6*$C$7^(A21-1)*IF(B21="Boss",$C$8,1),0)</f>
+        <f>ROUND(S21*IF(B21="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q21" s="16">
         <f>IF(O21&gt;=P21,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R21" s="18">
+        <f>INDEX($G$6:$G$11,INT((A21-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S21" s="18">
+        <f>S20*R21</f>
         <v/>
       </c>
     </row>
@@ -9401,11 +9644,19 @@
         <v/>
       </c>
       <c r="P22" s="18">
-        <f>ROUND($C$6*$C$7^(A22-1)*IF(B22="Boss",$C$8,1),0)</f>
+        <f>ROUND(S22*IF(B22="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q22" s="16">
         <f>IF(O22&gt;=P22,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R22" s="18">
+        <f>INDEX($G$6:$G$11,INT((A22-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S22" s="18">
+        <f>S21*R22</f>
         <v/>
       </c>
     </row>
@@ -9469,11 +9720,19 @@
         <v/>
       </c>
       <c r="P23" s="22">
-        <f>ROUND($C$6*$C$7^(A23-1)*IF(B23="Boss",$C$8,1),0)</f>
+        <f>ROUND(S23*IF(B23="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q23" s="20">
         <f>IF(O23&gt;=P23,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R23" s="22">
+        <f>INDEX($G$6:$G$11,INT((A23-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S23" s="22">
+        <f>S22*R23</f>
         <v/>
       </c>
     </row>
@@ -9537,11 +9796,19 @@
         <v/>
       </c>
       <c r="P24" s="18">
-        <f>ROUND($C$6*$C$7^(A24-1)*IF(B24="Boss",$C$8,1),0)</f>
+        <f>ROUND(S24*IF(B24="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q24" s="16">
         <f>IF(O24&gt;=P24,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R24" s="18">
+        <f>INDEX($G$6:$G$11,INT((A24-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S24" s="18">
+        <f>S23*R24</f>
         <v/>
       </c>
     </row>
@@ -9605,11 +9872,19 @@
         <v/>
       </c>
       <c r="P25" s="18">
-        <f>ROUND($C$6*$C$7^(A25-1)*IF(B25="Boss",$C$8,1),0)</f>
+        <f>ROUND(S25*IF(B25="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q25" s="16">
         <f>IF(O25&gt;=P25,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R25" s="18">
+        <f>INDEX($G$6:$G$11,INT((A25-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S25" s="18">
+        <f>S24*R25</f>
         <v/>
       </c>
     </row>
@@ -9673,11 +9948,19 @@
         <v/>
       </c>
       <c r="P26" s="18">
-        <f>ROUND($C$6*$C$7^(A26-1)*IF(B26="Boss",$C$8,1),0)</f>
+        <f>ROUND(S26*IF(B26="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q26" s="16">
         <f>IF(O26&gt;=P26,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R26" s="18">
+        <f>INDEX($G$6:$G$11,INT((A26-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S26" s="18">
+        <f>S25*R26</f>
         <v/>
       </c>
     </row>
@@ -9741,11 +10024,19 @@
         <v/>
       </c>
       <c r="P27" s="22">
-        <f>ROUND($C$6*$C$7^(A27-1)*IF(B27="Boss",$C$8,1),0)</f>
+        <f>ROUND(S27*IF(B27="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q27" s="20">
         <f>IF(O27&gt;=P27,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R27" s="22">
+        <f>INDEX($G$6:$G$11,INT((A27-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S27" s="22">
+        <f>S26*R27</f>
         <v/>
       </c>
     </row>
@@ -9809,11 +10100,19 @@
         <v/>
       </c>
       <c r="P28" s="18">
-        <f>ROUND($C$6*$C$7^(A28-1)*IF(B28="Boss",$C$8,1),0)</f>
+        <f>ROUND(S28*IF(B28="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q28" s="16">
         <f>IF(O28&gt;=P28,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>INDEX($G$6:$G$11,INT((A28-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S28" s="18">
+        <f>S27*R28</f>
         <v/>
       </c>
     </row>
@@ -9877,11 +10176,19 @@
         <v/>
       </c>
       <c r="P29" s="18">
-        <f>ROUND($C$6*$C$7^(A29-1)*IF(B29="Boss",$C$8,1),0)</f>
+        <f>ROUND(S29*IF(B29="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q29" s="16">
         <f>IF(O29&gt;=P29,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R29" s="18">
+        <f>INDEX($G$6:$G$11,INT((A29-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S29" s="18">
+        <f>S28*R29</f>
         <v/>
       </c>
     </row>
@@ -9945,11 +10252,19 @@
         <v/>
       </c>
       <c r="P30" s="18">
-        <f>ROUND($C$6*$C$7^(A30-1)*IF(B30="Boss",$C$8,1),0)</f>
+        <f>ROUND(S30*IF(B30="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q30" s="16">
         <f>IF(O30&gt;=P30,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R30" s="18">
+        <f>INDEX($G$6:$G$11,INT((A30-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S30" s="18">
+        <f>S29*R30</f>
         <v/>
       </c>
     </row>
@@ -10013,11 +10328,19 @@
         <v/>
       </c>
       <c r="P31" s="22">
-        <f>ROUND($C$6*$C$7^(A31-1)*IF(B31="Boss",$C$8,1),0)</f>
+        <f>ROUND(S31*IF(B31="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q31" s="20">
         <f>IF(O31&gt;=P31,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R31" s="22">
+        <f>INDEX($G$6:$G$11,INT((A31-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S31" s="22">
+        <f>S30*R31</f>
         <v/>
       </c>
     </row>
@@ -10081,11 +10404,19 @@
         <v/>
       </c>
       <c r="P32" s="18">
-        <f>ROUND($C$6*$C$7^(A32-1)*IF(B32="Boss",$C$8,1),0)</f>
+        <f>ROUND(S32*IF(B32="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q32" s="16">
         <f>IF(O32&gt;=P32,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R32" s="18">
+        <f>INDEX($G$6:$G$11,INT((A32-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S32" s="18">
+        <f>S31*R32</f>
         <v/>
       </c>
     </row>
@@ -10149,11 +10480,19 @@
         <v/>
       </c>
       <c r="P33" s="18">
-        <f>ROUND($C$6*$C$7^(A33-1)*IF(B33="Boss",$C$8,1),0)</f>
+        <f>ROUND(S33*IF(B33="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q33" s="16">
         <f>IF(O33&gt;=P33,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R33" s="18">
+        <f>INDEX($G$6:$G$11,INT((A33-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S33" s="18">
+        <f>S32*R33</f>
         <v/>
       </c>
     </row>
@@ -10217,11 +10556,19 @@
         <v/>
       </c>
       <c r="P34" s="18">
-        <f>ROUND($C$6*$C$7^(A34-1)*IF(B34="Boss",$C$8,1),0)</f>
+        <f>ROUND(S34*IF(B34="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q34" s="16">
         <f>IF(O34&gt;=P34,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R34" s="18">
+        <f>INDEX($G$6:$G$11,INT((A34-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S34" s="18">
+        <f>S33*R34</f>
         <v/>
       </c>
     </row>
@@ -10285,11 +10632,19 @@
         <v/>
       </c>
       <c r="P35" s="22">
-        <f>ROUND($C$6*$C$7^(A35-1)*IF(B35="Boss",$C$8,1),0)</f>
+        <f>ROUND(S35*IF(B35="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q35" s="20">
         <f>IF(O35&gt;=P35,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R35" s="22">
+        <f>INDEX($G$6:$G$11,INT((A35-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S35" s="22">
+        <f>S34*R35</f>
         <v/>
       </c>
     </row>
@@ -10353,11 +10708,19 @@
         <v/>
       </c>
       <c r="P36" s="18">
-        <f>ROUND($C$6*$C$7^(A36-1)*IF(B36="Boss",$C$8,1),0)</f>
+        <f>ROUND(S36*IF(B36="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q36" s="16">
         <f>IF(O36&gt;=P36,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R36" s="18">
+        <f>INDEX($G$6:$G$11,INT((A36-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S36" s="18">
+        <f>S35*R36</f>
         <v/>
       </c>
     </row>
@@ -10421,11 +10784,19 @@
         <v/>
       </c>
       <c r="P37" s="18">
-        <f>ROUND($C$6*$C$7^(A37-1)*IF(B37="Boss",$C$8,1),0)</f>
+        <f>ROUND(S37*IF(B37="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q37" s="16">
         <f>IF(O37&gt;=P37,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R37" s="18">
+        <f>INDEX($G$6:$G$11,INT((A37-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S37" s="18">
+        <f>S36*R37</f>
         <v/>
       </c>
     </row>
@@ -10489,11 +10860,19 @@
         <v/>
       </c>
       <c r="P38" s="18">
-        <f>ROUND($C$6*$C$7^(A38-1)*IF(B38="Boss",$C$8,1),0)</f>
+        <f>ROUND(S38*IF(B38="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q38" s="16">
         <f>IF(O38&gt;=P38,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R38" s="18">
+        <f>INDEX($G$6:$G$11,INT((A38-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S38" s="18">
+        <f>S37*R38</f>
         <v/>
       </c>
     </row>
@@ -10557,11 +10936,19 @@
         <v/>
       </c>
       <c r="P39" s="22">
-        <f>ROUND($C$6*$C$7^(A39-1)*IF(B39="Boss",$C$8,1),0)</f>
+        <f>ROUND(S39*IF(B39="Boss",$C$8,1),0)</f>
         <v/>
       </c>
       <c r="Q39" s="20">
         <f>IF(O39&gt;=P39,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="R39" s="22">
+        <f>INDEX($G$6:$G$11,INT((A39-1)/4)+1)</f>
+        <v/>
+      </c>
+      <c r="S39" s="22">
+        <f>S38*R39</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Hand size 8; threshold growth 1.5/2/2.5/3/3.25/3.5
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Morpheme_Master.xlsx
+++ b/Morpheme_Master.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Every round has a score threshold. It grows per round by a factor that rises in blocks of four rounds (1.5× for rounds 1–4, 2× for 5–8, 2.5× for 9–12, 3× for 13–16, 3.5× for 17–20, 5× for 21–24), with a ×3 bump on Boss Rounds. Missing one costs a life — the round is then replayed — or ends the run.</t>
+          <t>Every round has a score threshold. It grows per round by a factor that rises in blocks of four rounds (1.5× for rounds 1–4, 2× for 5–8, 2.5× for 9–12, 3× for 13–16, 3.25× for 17–20, 3.5× for 21–24), with a ×3 bump on Boss Rounds. Missing one costs a life — the round is then replayed — or ends the run.</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Implemented: 1.5 / 2 / 2.5 / 3 / 3.5 / 5 (Scoring tab G6:G11; editable live in the debug panel). Fallbacks to try if humans stall at B3–B4: 1.5/1.75/2/2.25/2.5/3.</t>
+          <t>Implemented: 1.5 / 2 / 2.5 / 3 / 3.25 / 3.5 (Scoring tab G6:G11; editable live in the debug panel). Softened from 3.5 / 5 in the last two blocks on 2026-09-18. Fallback if humans stall at B3–B4: 1.5/1.75/2/2.25/2.5/3.</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>Watch where humans stall; B4 = 2.05M and B6 = 192B need strong multiplier stacking.</t>
+          <t>Watch where humans stall; B4 = 2.05M, B6 = 34B. Hand size 10 → 8 at the same time.</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4274,7 +4273,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -4346,7 +4344,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -4742,7 +4739,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
@@ -8973,7 +8969,7 @@
         </is>
       </c>
       <c r="G10" s="15" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="11">
@@ -8991,7 +8987,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="12">
@@ -9016,11 +9012,11 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Tiles drawn each regular round (raised from 7). Not used by the formulas below; the engine reads it.</t>
+          <t>Tiles drawn each regular round (10 → 8 on 2026-09-18; Substrate adds more). Not used by the formulas below; the engine reads it.</t>
         </is>
       </c>
     </row>

</xml_diff>